<commit_message>
Prioritize dynastic costume and military dramas in English2 reschedule
</commit_message>
<xml_diff>
--- a/schedules/english2_20261105_20261115_costume/english2_schedule_20261105_20261115.xlsx
+++ b/schedules/english2_20261105_20261115_costume/english2_schedule_20261105_20261115.xlsx
@@ -17,13 +17,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="完整排片更新表" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英语2每日一部'!$A$1:$P$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'英语2每日一部'!$A$1:$Q$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'跨频道7天核验'!$A$1:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'被替换的原安排'!$A$1:$E$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'英语2历史去重'!$A$1:$C$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'古装候选池'!$A$1:$H$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'古装候选池'!$A$1:$H$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'排除剧目'!$A$1:$I$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排片说明'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'排片说明'!$A$1:$B$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -462,14 +462,15 @@
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,50 +506,55 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>题材优先级</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>英语配音标记</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>出剧日期</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>资源表工作表</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>资源表行号</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>英语2历史去重</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>外采代运营禁播筛查</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>跨频道最小间隔/小时</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>publish_local</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>publish_at</t>
         </is>
@@ -572,61 +578,66 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>我剑即天威</t>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026 WW60</t>
+          <t>2026 WW27</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>古装修仙剑道</t>
+          <t>古代边疆军旅</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>优先：王朝权谋或军旅</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
-        <v>1043</v>
-      </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="2" t="n">
+        <v>964</v>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
-        <v>253</v>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2026-11-05T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>2026-11-05T05:00:00Z</t>
         </is>
@@ -665,48 +676,53 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>其次：古装江湖或宫廷奇幻</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>1038</v>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>无同剧记录</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>2026-11-06T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>2026-11-06T05:00:00Z</t>
         </is>
@@ -730,61 +746,68 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>武魂觉醒我用锤子一人成军</t>
+          <t>百岁剑仙被千金倒追了</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026 WW52</t>
+          <t>2026 WW38</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>古装武魂与机械兽</t>
+          <t>古代剑仙江湖</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>其次：古装江湖或宫廷奇幻</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
-        <v>1019</v>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="2" t="n">
+        <v>976</v>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
-        <v>349</v>
-      </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
+          <t>无同剧记录</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
           <t>2026-11-07T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>2026-11-07T05:00:00Z</t>
         </is>
@@ -808,61 +831,66 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>被换灵骨后我成了大帝</t>
+          <t>我剑即天威</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026 WW48</t>
+          <t>2026 WW60</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>古装剑道修仙</t>
+          <t>古装修仙剑道</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>补足：古装仙侠玄幻</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n">
-        <v>1009</v>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="L5" s="2" t="n">
+        <v>1043</v>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N5" s="2" t="n">
-        <v>349</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="n">
+        <v>325</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>2026-11-08T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>2026-11-08T05:00:00Z</t>
         </is>
@@ -886,63 +914,66 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>百岁剑仙被千金倒追了</t>
+          <t>被换灵骨后我成了大帝</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026 WW38</t>
+          <t>2026 WW48</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>古代剑仙江湖</t>
+          <t>古装剑道修仙</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>补足：古装仙侠玄幻</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n">
-        <v>976</v>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="L6" s="2" t="n">
+        <v>1009</v>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>无同剧记录</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="n">
+        <v>373</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>2026-11-09T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>2026-11-09T05:00:00Z</t>
         </is>
@@ -966,61 +997,66 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
+          <t>我一邪修养反派为徒很正常吧</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026 WW27</t>
+          <t>2026 WW26</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>古代边疆军旅</t>
+          <t>古装修仙宗门</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>补足：古装仙侠玄幻</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n">
-        <v>964</v>
-      </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L7" s="2" t="n">
+        <v>957</v>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N7" s="2" t="n">
+      <c r="O7" s="2" t="n">
         <v>493</v>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>2026-11-10T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>2026-11-10T05:00:00Z</t>
         </is>
@@ -1044,61 +1080,66 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>我一邪修养反派为徒很正常吧</t>
+          <t>厨神帝王录</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026 WW26</t>
+          <t>2609 KR20</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>古装修仙宗门</t>
+          <t>古代王朝权谋</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>优先：王朝权谋或军旅</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>未填；剧集代码标2026年</t>
-        </is>
-      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n">
-        <v>957</v>
-      </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="L8" s="2" t="n">
+        <v>685</v>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
-        <v>517</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>2026-11-11T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>2026-11-11T05:00:00Z</t>
         </is>
@@ -1122,61 +1163,66 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>元始我申公豹请你上榜封神</t>
+          <t>大明憨王爹我真想就藩</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2609 KR78</t>
+          <t>2026 WW73</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>古装封神神话</t>
+          <t>明代历史穿越与赈灾军旅</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
+          <t>优先：王朝权谋或军旅</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
+          <t>未填；剧集代码标2026年</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n">
-        <v>836</v>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="L9" s="2" t="n">
+        <v>1110</v>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
-        <v>380</v>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O9" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>2026-11-12T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>2026-11-12T05:00:00Z</t>
         </is>
@@ -1200,61 +1246,66 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>你退你的婚我撩我的师尊</t>
+          <t>元始我申公豹请你上榜封神</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2609 KR74</t>
+          <t>2609 KR78</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>古装修仙师徒</t>
+          <t>古装封神神话</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
+          <t>补足：古装仙侠玄幻</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n">
-        <v>820</v>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="L10" s="2" t="n">
+        <v>836</v>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
-        <v>805</v>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="n">
+        <v>404</v>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>2026-11-13T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>2026-11-13T05:00:00Z</t>
         </is>
@@ -1293,46 +1344,51 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
+          <t>其次：古装江湖或宫廷奇幻</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>762</v>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="O11" s="2" t="n">
         <v>176</v>
       </c>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>2026-11-14T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>2026-11-14T05:00:00Z</t>
         </is>
@@ -1356,68 +1412,73 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>万倍返还弟子越强我越神</t>
+          <t>你退你的婚我撩我的师尊</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2609 KR44</t>
+          <t>2609 KR74</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>古装修仙宗门</t>
+          <t>古装修仙师徒</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
+          <t>补足：古装仙侠玄幻</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
           <t>最新剧集</t>
         </is>
       </c>
-      <c r="K12" s="2" t="n">
-        <v>760</v>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L12" s="2" t="n">
+        <v>820</v>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="N12" s="3" t="inlineStr">
         <is>
           <t>通过</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
-        <v>181</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="n">
+        <v>853</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>2026-11-15T13:00:00+08:00</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>2026-11-15T05:00:00Z</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P12"/>
+  <autoFilter ref="A1:Q12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1467,7 +1528,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>我剑即天威</t>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -1477,7 +1538,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-25T00:00:00+08:00~2026-10-25T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
+          <t>2026-10-14T00:00:00+08:00~2026-10-14T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）；2026-10-15T00:00:00+08:00~2026-10-15T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 俄语 最新排片表（空白表头顺延）；2026-10-20T17:00:00+08:00~2026-10-20T17:00:00+08:00 俄语 已交付程序排期</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1572,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>武魂觉醒我用锤子一人成军</t>
+          <t>百岁剑仙被千金倒追了</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1521,7 +1582,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T00:00:00+08:00~2026-09-28T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-17T00:00:00+08:00~2026-10-17T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）；2026-10-23T00:00:00+08:00~2026-10-23T23:59:59.999999+08:00 俄语 最新排片表（空白表头顺延）；2026-10-23T17:00:00+08:00~2026-10-23T17:00:00+08:00 俄语 已交付程序排期</t>
+          <t>无同剧记录</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1594,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>被换灵骨后我成了大帝</t>
+          <t>我剑即天威</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1543,7 +1604,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24T00:00:00+08:00~2026-10-24T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
+          <t>2026-10-25T00:00:00+08:00~2026-10-25T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1616,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>百岁剑仙被千金倒追了</t>
+          <t>被换灵骨后我成了大帝</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1565,7 +1626,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>无同剧记录</t>
+          <t>2026-10-24T00:00:00+08:00~2026-10-24T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1638,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
+          <t>我一邪修养反派为徒很正常吧</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1587,7 +1648,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T00:00:00+08:00~2026-10-14T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）；2026-10-15T00:00:00+08:00~2026-10-15T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 俄语 最新排片表（空白表头顺延）；2026-10-20T17:00:00+08:00~2026-10-20T17:00:00+08:00 俄语 已交付程序排期</t>
+          <t>2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1660,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>我一邪修养反派为徒很正常吧</t>
+          <t>厨神帝王录</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1609,7 +1670,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
+          <t>2026-11-03T17:00:00+08:00~2026-11-03T17:00:00+08:00 英语1 已交付程序排期</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1682,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>元始我申公豹请你上榜封神</t>
+          <t>大明憨王爹我真想就藩</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1631,7 +1692,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T00:00:00+08:00~2026-10-06T23:59:59.999999+08:00 西语 最新排片表（空白表头顺延）；2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-27T17:00:00+08:00~2026-10-27T17:00:00+08:00 英语1 已交付程序排期</t>
+          <t>2026-11-05T12:00:00+08:00~2026-11-05T12:00:00+08:00 菲律宾语 10月30日调整菲律宾语排片</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1704,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>你退你的婚我撩我的师尊</t>
+          <t>元始我申公豹请你上榜封神</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1653,7 +1714,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T00:00:00+08:00~2026-10-02T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-10T00:00:00+08:00~2026-10-10T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
+          <t>2026-10-06T00:00:00+08:00~2026-10-06T23:59:59.999999+08:00 西语 最新排片表（空白表头顺延）；2026-10-20T00:00:00+08:00~2026-10-20T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-27T17:00:00+08:00~2026-10-27T17:00:00+08:00 英语1 已交付程序排期</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1748,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>万倍返还弟子越强我越神</t>
+          <t>你退你的婚我撩我的师尊</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1697,7 +1758,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18T00:00:00+08:00~2026-10-18T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）；2026-11-07T00:00:00+08:00~2026-11-07T23:59:59.999999+08:00 俄语 最新排片表（空白表头顺延）；2026-11-07T17:00:00+08:00~2026-11-07T17:00:00+08:00 俄语 已交付程序排期</t>
+          <t>2026-10-02T00:00:00+08:00~2026-10-02T23:59:59.999999+08:00 韩语 最新排片表（空白表头顺延）；2026-10-10T00:00:00+08:00~2026-10-10T23:59:59.999999+08:00 英语1 最新排片表（空白表头顺延）</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1829,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>我剑即天威</t>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026 WW60</t>
+          <t>2026 WW27</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -2302,7 +2363,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>备选</t>
+          <t>已选</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2483,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>已选</t>
+          <t>备选</t>
         </is>
       </c>
     </row>
@@ -2469,17 +2530,17 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>你退你的婚我撩我的师尊</t>
+          <t>不当黄牛全族发愁</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2609 KR74</t>
+          <t>2609 KR56</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>古装修仙师徒</t>
+          <t>古代乡土与科举</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2489,7 +2550,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>有</t>
+          <t>有/新</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2498,28 +2559,28 @@
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>820</v>
+        <v>786</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>已选</t>
+          <t>7天间隔内无可用位置</t>
         </is>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>元始我申公豹请你上榜封神</t>
+          <t>只想种地扶贫奈何万民归顺</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2609 KR78</t>
+          <t>2609 KR66</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>古装封神神话</t>
+          <t>古代王朝农业与权谋</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -2538,28 +2599,28 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>836</v>
+        <v>803</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>已选</t>
+          <t>7天间隔内无可用位置</t>
         </is>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>旁人笑我木讷不知我有老仙金手指</t>
+          <t>你退你的婚我撩我的师尊</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2609 KR82</t>
+          <t>2609 KR74</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>古装修仙宗门</t>
+          <t>古装修仙师徒</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -2569,7 +2630,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>有/新</t>
+          <t>有</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2578,28 +2639,28 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>848</v>
+        <v>820</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>7天间隔内无可用位置</t>
+          <t>已选</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>穿越女频开局送皇后白月光进东厂</t>
+          <t>元始我申公豹请你上榜封神</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2609 KR85</t>
+          <t>2609 KR78</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>古代宫廷穿越</t>
+          <t>古装封神神话</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2618,28 +2679,28 @@
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>863</v>
+        <v>836</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>7天间隔内无可用位置</t>
+          <t>已选</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>我宗门真的全是老弱病残啊</t>
+          <t>旁人笑我木讷不知我有老仙金手指</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2609 KR87</t>
+          <t>2609 KR82</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>古装武道宗门</t>
+          <t>古装修仙宗门</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -2649,16 +2710,16 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>有</t>
+          <t>有/新</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>873</v>
+        <v>848</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -2669,17 +2730,17 @@
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>我一邪修养反派为徒很正常吧</t>
+          <t>穿越女频开局送皇后白月光进东厂</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026 WW26</t>
+          <t>2609 KR85</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>古装修仙宗门</t>
+          <t>古代宫廷穿越</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -2694,32 +2755,32 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>未填；剧集代码标2026年</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>957</v>
+        <v>863</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>已选</t>
+          <t>7天间隔内无可用位置</t>
         </is>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
+          <t>我宗门真的全是老弱病残啊</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026 WW27</t>
+          <t>2609 KR87</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>古代边疆军旅</t>
+          <t>古装武道宗门</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2734,32 +2795,32 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>未填；剧集代码标2026年</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>964</v>
+        <v>873</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>已选</t>
+          <t>7天间隔内无可用位置</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>百岁剑仙被千金倒追了</t>
+          <t>我一邪修养反派为徒很正常吧</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2026 WW38</t>
+          <t>2026 WW26</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>古代剑仙江湖</t>
+          <t>古装修仙宗门</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -2778,7 +2839,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>976</v>
+        <v>957</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -2789,17 +2850,17 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>被换灵骨后我成了大帝</t>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026 WW48</t>
+          <t>2026 WW27</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>古装剑道修仙</t>
+          <t>古代边疆军旅</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -2818,7 +2879,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>1009</v>
+        <v>964</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -2829,17 +2890,17 @@
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>武魂觉醒我用锤子一人成军</t>
+          <t>百岁剑仙被千金倒追了</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026 WW52</t>
+          <t>2026 WW38</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>古装武魂与机械兽</t>
+          <t>古代剑仙江湖</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -2858,7 +2919,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1019</v>
+        <v>976</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -2869,17 +2930,17 @@
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>驴神归来时速八百</t>
+          <t>被换灵骨后我成了大帝</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026 WW56</t>
+          <t>2026 WW48</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>古代战神重生</t>
+          <t>古装剑道修仙</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2898,7 +2959,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1038</v>
+        <v>1009</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -2909,45 +2970,165 @@
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>武魂觉醒我用锤子一人成军</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW52</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>古装武魂与机械兽</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>男频</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>有</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>未填；剧集代码标2026年</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1019</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>备选</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>驴神归来时速八百</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW56</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>古代战神重生</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>男频</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>有</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>未填；剧集代码标2026年</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1038</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>已选</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>我剑即天威</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>2026 WW60</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>古装修仙剑道</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>男频</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>有</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>未填；剧集代码标2026年</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>1043</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>已选</t>
         </is>
       </c>
     </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>大明憨王爹我真想就藩</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW73</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>明代历史穿越与赈灾军旅</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>男频</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>有</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>未填；剧集代码标2026年</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1110</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>已选</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H21"/>
+  <autoFilter ref="A1:H24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4486,7 +4667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4508,113 +4689,125 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>范围与时间</t>
+          <t>古装优先重排</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026年11月5—15日，每天北京时间13:00一部，共11部。沿用英语2原发布时间13:00，截止日沿用此前11月15日。</t>
+          <t>根据用户再次要求，王朝权谋、历史穿越、边疆军旅优先，其次古装江湖与宫廷奇幻，再用古装仙侠补足；本版移除机械兽题材。纯王朝类受历史去重与7天间隔限制不足11部，已在明细标注题材优先级。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>改动范围</t>
+          <t>范围与时间</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>英语2的11月5日起重新安排，11月4日及之前不动。其他频道所有单元格保持最新已交付排片不变，包括10月30日调整后的菲律宾语22部。</t>
+          <t>2026年11月5—15日，每天北京时间13:00一部，共11部。沿用英语2原发布时间13:00，截止日沿用此前11月15日。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>被替换安排</t>
+          <t>改动范围</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>原英语2 11月5日《开局成破剑竟被她进化成神兵》、11月6日《代号枪神》替换；这两部仍计入英语2去重，不复用。</t>
+          <t>英语2的11月5日起重新安排，11月4日及之前不动。其他频道所有单元格保持最新已交付排片不变，包括10月30日调整后的菲律宾语22部。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>题材与语种</t>
+          <t>被替换安排</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>本次11部全部为根据简介核对的古代王朝、古装江湖或仙侠玄幻背景，均为资源表明确男频、英语栏标有或有/新。机械兽等元素属于古装玄幻混合题材，已单列背景。</t>
+          <t>原英语2 11月5日《开局成破剑竟被她进化成神兵》、11月6日《代号枪神》替换；这两部仍计入英语2去重，不复用。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>严格排除</t>
+          <t>题材与语种</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>同剧任一版本文字标注外采、代运营或禁播即排除；不把外采-解禁慢当作可用片源。沿用此前用户要求按文字标记核验。</t>
+          <t>本次11部全部为根据简介核对的古代王朝、古装江湖或仙侠玄幻背景，均为资源表明确男频、英语栏标有或有/新。本版不含机械兽混合题材；宫廷修仙、神话及其他仙侠仍有超自然设定，已逐部标注。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>历史去重与异名</t>
+          <t>严格排除</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>英语2现有14个剧目全避用；《剑道巅峰从一把锈剑开始》按《开局成破剑竟被她进化成神兵》的同类异名剧情保守排除，避免变更片名后重复。</t>
+          <t>同剧任一版本文字标注外采、代运营或禁播即排除；不把外采-解禁慢当作可用片源。沿用此前用户要求按文字标记核验。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>跨频道间隔</t>
+          <t>历史去重与异名</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>与上传排片、已交付后续排期及菲律宾语10月30日新版核对至少168小时，最短176小时。仅知日期的记录按全天范围计算；近似同剧情异名亦保守计入。无法核验未提供的Studio线上变更。</t>
+          <t>英语2现有14个剧目全避用；《剑道巅峰从一把锈剑开始》按《开局成破剑竟被她进化成神兵》的同类异名剧情保守排除，避免变更片名后重复。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>日期信息</t>
+          <t>跨频道间隔</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026 WW片源具体出剧日期未填，只能确认代码标2026年，不据此宣称某月新剧；其余KR片源有2026年明确出剧日期。</t>
+          <t>与上传排片、已交付后续排期及菲律宾语10月30日新版核对至少168小时，最短176小时。仅知日期的记录按全天范围计算；近似同剧情异名亦保守计入。无法核验未提供的Studio线上变更。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>日期信息</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026 WW片源具体出剧日期未填，只能确认代码标2026年，不据此宣称某月新剧；其余KR片源有2026年明确出剧日期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>交付范围</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>本次只排片，不制作标题封面、不改原程序素材、不修改飞书或YouTube。若原11月5—6日已在Studio定时，需自行调整；下载排片不会取消线上旧定时。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6146,57 +6339,57 @@
       </c>
       <c r="AZ7" s="2" t="inlineStr">
         <is>
+          <t>边疆老卒御赐老婆后我越活越勇</t>
+        </is>
+      </c>
+      <c r="BA7" s="2" t="inlineStr">
+        <is>
+          <t>驴神归来时速八百</t>
+        </is>
+      </c>
+      <c r="BB7" s="2" t="inlineStr">
+        <is>
+          <t>百岁剑仙被千金倒追了</t>
+        </is>
+      </c>
+      <c r="BC7" s="2" t="inlineStr">
+        <is>
           <t>我剑即天威</t>
         </is>
       </c>
-      <c r="BA7" s="2" t="inlineStr">
-        <is>
-          <t>驴神归来时速八百</t>
-        </is>
-      </c>
-      <c r="BB7" s="2" t="inlineStr">
-        <is>
-          <t>武魂觉醒我用锤子一人成军</t>
-        </is>
-      </c>
-      <c r="BC7" s="2" t="inlineStr">
+      <c r="BD7" s="2" t="inlineStr">
         <is>
           <t>被换灵骨后我成了大帝</t>
         </is>
       </c>
-      <c r="BD7" s="2" t="inlineStr">
-        <is>
-          <t>百岁剑仙被千金倒追了</t>
-        </is>
-      </c>
       <c r="BE7" s="2" t="inlineStr">
         <is>
-          <t>边疆老卒御赐老婆后我越活越勇</t>
+          <t>我一邪修养反派为徒很正常吧</t>
         </is>
       </c>
       <c r="BF7" s="2" t="inlineStr">
         <is>
-          <t>我一邪修养反派为徒很正常吧</t>
+          <t>厨神帝王录</t>
         </is>
       </c>
       <c r="BG7" s="2" t="inlineStr">
         <is>
+          <t>大明憨王爹我真想就藩</t>
+        </is>
+      </c>
+      <c r="BH7" s="2" t="inlineStr">
+        <is>
           <t>元始我申公豹请你上榜封神</t>
         </is>
       </c>
-      <c r="BH7" s="2" t="inlineStr">
+      <c r="BI7" s="2" t="inlineStr">
+        <is>
+          <t>太监从后宫签到成圣</t>
+        </is>
+      </c>
+      <c r="BJ7" s="2" t="inlineStr">
         <is>
           <t>你退你的婚我撩我的师尊</t>
-        </is>
-      </c>
-      <c r="BI7" s="2" t="inlineStr">
-        <is>
-          <t>太监从后宫签到成圣</t>
-        </is>
-      </c>
-      <c r="BJ7" s="2" t="inlineStr">
-        <is>
-          <t>万倍返还弟子越强我越神</t>
         </is>
       </c>
     </row>

</xml_diff>